<commit_message>
fix: event subcription dangling, leaking in texture and global set flip vertically on load
</commit_message>
<xml_diff>
--- a/docs/testcases/axis_engine_testcases.xlsx
+++ b/docs/testcases/axis_engine_testcases.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Re27325da939a4b24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestCases" sheetId="2" r:id="Rd5f83af73aef4706"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AutomatedTests" sheetId="3" r:id="R0cdd887403084030"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ExecutionPlan" sheetId="4" r:id="Rda659c1ddc1b44b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R2b8f2e6e4d1c4715"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestCases" sheetId="2" r:id="R56b42b9b18b840ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AutomatedTests" sheetId="3" r:id="Re51f4bb6cac44d19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ExecutionPlan" sheetId="4" r:id="R9a40ae47156f40f5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -254,7 +254,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="21.25" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="27.5" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="65" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="2.5" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="21.25" hidden="0" customWidth="1"/>
@@ -317,21 +317,18 @@
         <x:v>Total testcases</x:v>
       </x:c>
       <x:c r="B4" t="n">
-        <x:f>COUNTA(TestCases!A2:A200)</x:f>
-        <x:v>74</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="D4" t="str">
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E4" t="n">
-        <x:f>COUNTIF(TestCases!K2:K200,D4)</x:f>
-        <x:v>24</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="G4" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H4" t="n">
-        <x:f>COUNTIF(TestCases!B2:B200,G4)</x:f>
         <x:v>46</x:v>
       </x:c>
     </x:row>
@@ -340,22 +337,19 @@
         <x:v>Implemented automated</x:v>
       </x:c>
       <x:c r="B5" t="n">
-        <x:f>COUNTIF(TestCases!K2:K200,"Implemented")</x:f>
-        <x:v>24</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="D5" t="str">
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="E5" t="n">
-        <x:f>COUNTIF(TestCases!K2:K200,D5)</x:f>
         <x:v>34</x:v>
       </x:c>
       <x:c r="G5" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="H5" t="n">
-        <x:f>COUNTIF(TestCases!B2:B200,G5)</x:f>
-        <x:v>26</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -363,22 +357,19 @@
         <x:v>Planned automated</x:v>
       </x:c>
       <x:c r="B6" t="n">
-        <x:f>COUNTIF(TestCases!K2:K200,"Planned")</x:f>
         <x:v>34</x:v>
       </x:c>
       <x:c r="D6" t="str">
         <x:v>Manual</x:v>
       </x:c>
       <x:c r="E6" t="n">
-        <x:f>COUNTIF(TestCases!K2:K200,D6)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="G6" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="H6" t="n">
-        <x:f>COUNTIF(TestCases!B2:B200,G6)</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -393,7 +384,6 @@
         <x:v>Manual/Expected-Fail</x:v>
       </x:c>
       <x:c r="E7" t="n">
-        <x:f>COUNTIF(TestCases!K2:K200,D7)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="G7" t="str"/>
@@ -411,7 +401,6 @@
         <x:v>Planned/Bug</x:v>
       </x:c>
       <x:c r="E8" t="n">
-        <x:f>COUNTIF(TestCases!K2:K200,D8)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="G8" t="str"/>
@@ -422,7 +411,7 @@
         <x:v>Generated from source review</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>2026-06-05</x:v>
+        <x:v>2026-06-06</x:v>
       </x:c>
       <x:c r="D9" t="str"/>
       <x:c r="E9" t="str"/>
@@ -432,7 +421,7 @@
         <x:v>Test executable</x:v>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>build\bin\axis_engine_tests.exe</x:v>
+        <x:v>build\bin\axis_test.exe</x:v>
       </x:c>
       <x:c r="D10" t="str"/>
       <x:c r="E10" t="str"/>
@@ -514,7 +503,7 @@
         <x:v>Command</x:v>
       </x:c>
       <x:c r="B18" s="9" t="str">
-        <x:v>cmake --build build --config Debug --target axis_engine_tests</x:v>
+        <x:v>cmake --build build --config Debug --target axis_test</x:v>
       </x:c>
       <x:c r="C18" s="9" t="str"/>
       <x:c r="D18" s="9" t="str"/>
@@ -528,7 +517,7 @@
         <x:v>Command</x:v>
       </x:c>
       <x:c r="B19" s="9" t="str">
-        <x:v>build\bin\axis_engine_tests.exe</x:v>
+        <x:v>build\bin\axis_test.exe</x:v>
       </x:c>
       <x:c r="C19" s="9" t="str"/>
       <x:c r="D19" s="9" t="str"/>
@@ -3705,6 +3694,267 @@
         <x:v>Audio manual regression.</x:v>
       </x:c>
     </x:row>
+    <x:row r="76">
+      <x:c r="A76" t="str">
+        <x:v>EV-001</x:v>
+      </x:c>
+      <x:c r="B76" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C76" t="str">
+        <x:v>Unit</x:v>
+      </x:c>
+      <x:c r="D76" t="str">
+        <x:v>Core/EventManager</x:v>
+      </x:c>
+      <x:c r="E76" t="str">
+        <x:v>include/engine/core/logic/event_manager.h</x:v>
+      </x:c>
+      <x:c r="F76" t="str">
+        <x:v>Generic unsubscribe removes listener across event dispatchers</x:v>
+      </x:c>
+      <x:c r="G76" t="str">
+        <x:v>A listener is subscribed to an event and only the numeric listener id is retained.</x:v>
+      </x:c>
+      <x:c r="H76" t="str">
+        <x:v>1. Subscribe listener.
+2. Publish once and verify callback runs.
+3. Call EventManager::Unsubscribe(id).
+4. Publish again.</x:v>
+      </x:c>
+      <x:c r="I76" t="str">
+        <x:v>TestEvent value=1</x:v>
+      </x:c>
+      <x:c r="J76" t="str">
+        <x:v>Callback is removed and no dangling callback fires after generic unsubscribe.</x:v>
+      </x:c>
+      <x:c r="K76" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+      <x:c r="L76" t="str">
+        <x:v>tests/unit/test_event_manager.cpp</x:v>
+      </x:c>
+      <x:c r="M76" t="str">
+        <x:v>Regression for system callbacks that store only listener ids.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" t="str">
+        <x:v>EV-002</x:v>
+      </x:c>
+      <x:c r="B77" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C77" t="str">
+        <x:v>Unit</x:v>
+      </x:c>
+      <x:c r="D77" t="str">
+        <x:v>Core/EventSubscriptionList</x:v>
+      </x:c>
+      <x:c r="E77" t="str">
+        <x:v>include/engine/core/logic/event_manager.h</x:v>
+      </x:c>
+      <x:c r="F77" t="str">
+        <x:v>Subscription list clears mixed event types</x:v>
+      </x:c>
+      <x:c r="G77" t="str">
+        <x:v>Two different event types have active subscriptions stored in one EventSubscriptionList.</x:v>
+      </x:c>
+      <x:c r="H77" t="str">
+        <x:v>1. Add both listener ids to EventSubscriptionList.
+2. Publish both events.
+3. Clear list.
+4. Publish both events again.</x:v>
+      </x:c>
+      <x:c r="I77" t="str">
+        <x:v>TestEventA/TestEventB</x:v>
+      </x:c>
+      <x:c r="J77" t="str">
+        <x:v>Both callbacks stop firing after Clear(), covering system Shutdown() cleanup.</x:v>
+      </x:c>
+      <x:c r="K77" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+      <x:c r="L77" t="str">
+        <x:v>tests/unit/test_event_manager.cpp</x:v>
+      </x:c>
+      <x:c r="M77" t="str">
+        <x:v>Regression for dangling system callbacks after destroy/reinitialize.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" t="str">
+        <x:v>TX-001</x:v>
+      </x:c>
+      <x:c r="B78" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C78" t="str">
+        <x:v>Unit</x:v>
+      </x:c>
+      <x:c r="D78" t="str">
+        <x:v>Render/Texture</x:v>
+      </x:c>
+      <x:c r="E78" t="str">
+        <x:v>include/engine/render/type/graphics_types.h</x:v>
+      </x:c>
+      <x:c r="F78" t="str">
+        <x:v>Pixel data ownership survives value copies</x:v>
+      </x:c>
+      <x:c r="G78" t="str">
+        <x:v>Texture owns CPU pixel bytes through SetPixelDataCopy.</x:v>
+      </x:c>
+      <x:c r="H78" t="str">
+        <x:v>1. Copy Texture by value.
+2. Release original CPU data.
+3. Inspect copied Texture.</x:v>
+      </x:c>
+      <x:c r="I78" t="str">
+        <x:v>RGBA bytes {1,2,3,4}</x:v>
+      </x:c>
+      <x:c r="J78" t="str">
+        <x:v>Copied Texture keeps valid pixelData and ownership; original releases cleanly.</x:v>
+      </x:c>
+      <x:c r="K78" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+      <x:c r="L78" t="str">
+        <x:v>tests/unit/test_texture_ownership.cpp</x:v>
+      </x:c>
+      <x:c r="M78" t="str">
+        <x:v>Regression for raw pixelData leaks/dangling pointers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" t="str">
+        <x:v>TX-002</x:v>
+      </x:c>
+      <x:c r="B79" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C79" t="str">
+        <x:v>Unit</x:v>
+      </x:c>
+      <x:c r="D79" t="str">
+        <x:v>Render/Texture</x:v>
+      </x:c>
+      <x:c r="E79" t="str">
+        <x:v>include/engine/render/type/graphics_types.h</x:v>
+      </x:c>
+      <x:c r="F79" t="str">
+        <x:v>Pixel data ownership survives vector reallocation</x:v>
+      </x:c>
+      <x:c r="G79" t="str">
+        <x:v>A vector stores Textures that own CPU pixel data.</x:v>
+      </x:c>
+      <x:c r="H79" t="str">
+        <x:v>1. Push multiple owned Textures into vector.
+2. Force vector value copies/moves.
+3. Inspect stored pixelData.</x:v>
+      </x:c>
+      <x:c r="I79" t="str">
+        <x:v>Two 1x1 RGBA buffers</x:v>
+      </x:c>
+      <x:c r="J79" t="str">
+        <x:v>Every stored Texture still owns valid pixelData after reallocation.</x:v>
+      </x:c>
+      <x:c r="K79" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+      <x:c r="L79" t="str">
+        <x:v>tests/unit/test_texture_ownership.cpp</x:v>
+      </x:c>
+      <x:c r="M79" t="str">
+        <x:v>Regression for Model/ResourceManager texture vectors.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" t="str">
+        <x:v>TX-003</x:v>
+      </x:c>
+      <x:c r="B80" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C80" t="str">
+        <x:v>Unit</x:v>
+      </x:c>
+      <x:c r="D80" t="str">
+        <x:v>Resource/TextureManager</x:v>
+      </x:c>
+      <x:c r="E80" t="str">
+        <x:v>src/resource/logic/texture_manager.cpp</x:v>
+      </x:c>
+      <x:c r="F80" t="str">
+        <x:v>Unload releases kept CPU pixel data</x:v>
+      </x:c>
+      <x:c r="G80" t="str">
+        <x:v>TextureManager creates a texture with keepCpuData=true.</x:v>
+      </x:c>
+      <x:c r="H80" t="str">
+        <x:v>1. Create texture from CPU bytes.
+2. Verify pixelData is owned.
+3. Call Unload(name).
+4. Inspect texture and fake low-level delete count.</x:v>
+      </x:c>
+      <x:c r="I80" t="str">
+        <x:v>1x1 RGBA buffer</x:v>
+      </x:c>
+      <x:c r="J80" t="str">
+        <x:v>CPU pixelData is released and GPU texture delete is requested once.</x:v>
+      </x:c>
+      <x:c r="K80" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+      <x:c r="L80" t="str">
+        <x:v>tests/unit/test_texture_ownership.cpp</x:v>
+      </x:c>
+      <x:c r="M80" t="str">
+        <x:v>Regression for hot reload/repeated load RAM leaks.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" t="str">
+        <x:v>BS-001</x:v>
+      </x:c>
+      <x:c r="B81" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="C81" t="str">
+        <x:v>Integration</x:v>
+      </x:c>
+      <x:c r="D81" t="str">
+        <x:v>Scene/BinarySceneSerializer</x:v>
+      </x:c>
+      <x:c r="E81" t="str">
+        <x:v>src/scene/logic/binary_scene_serializer.cpp</x:v>
+      </x:c>
+      <x:c r="F81" t="str">
+        <x:v>Binary serializer v3 round-trips config and material fields</x:v>
+      </x:c>
+      <x:c r="G81" t="str">
+        <x:v>Scene contains config values, material descriptor strings, camera and light components.</x:v>
+      </x:c>
+      <x:c r="H81" t="str">
+        <x:v>1. Save scene to binary file.
+2. Load into a new Scene.
+3. Inspect ConfigManager snapshot and loaded components.</x:v>
+      </x:c>
+      <x:c r="I81" t="str">
+        <x:v>strictAssetLoading, ambientIntensity, UI reference size, solverIterations, lightingMode</x:v>
+      </x:c>
+      <x:c r="J81" t="str">
+        <x:v>All v3 fields round-trip without raw struct layout dependency for tested config/material/camera/light fields.</x:v>
+      </x:c>
+      <x:c r="K81" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+      <x:c r="L81" t="str">
+        <x:v>tests/integration/test_binary_scene_serializer.cpp</x:v>
+      </x:c>
+      <x:c r="M81" t="str">
+        <x:v>Regression for missing config fields and raw material descriptor bytes.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:M1"/>
@@ -3720,8 +3970,8 @@
     <x:col min="1" max="1" width="11.25" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="23.75" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="45" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="32.5" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="65" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="37.5" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="70" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -3772,7 +4022,7 @@
         <x:v>tests/unit/test_yaml_parser.cpp</x:v>
       </x:c>
       <x:c r="E3" s="9" t="str">
-        <x:v>cmake --build build --config Debug --target axis_engine_tests &amp;&amp; build\bin\axis_engine_tests.exe</x:v>
+        <x:v>cmake --build build --config Debug --target axis_test &amp;&amp; build\bin\axis_test.exe</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -3789,7 +4039,7 @@
         <x:v>tests/unit/test_yaml_parser.cpp</x:v>
       </x:c>
       <x:c r="E4" s="9" t="str">
-        <x:v>cmake --build build --config Debug --target axis_engine_tests &amp;&amp; build\bin\axis_engine_tests.exe</x:v>
+        <x:v>cmake --build build --config Debug --target axis_test &amp;&amp; build\bin\axis_test.exe</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -3806,7 +4056,7 @@
         <x:v>tests/unit/test_yaml_parser.cpp</x:v>
       </x:c>
       <x:c r="E5" s="9" t="str">
-        <x:v>cmake --build build --config Debug --target axis_engine_tests &amp;&amp; build\bin\axis_engine_tests.exe</x:v>
+        <x:v>cmake --build build --config Debug --target axis_test &amp;&amp; build\bin\axis_test.exe</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -3823,7 +4073,7 @@
         <x:v>tests/unit/test_pathfinding.cpp</x:v>
       </x:c>
       <x:c r="E6" s="9" t="str">
-        <x:v>cmake --build build --config Debug --target axis_engine_tests &amp;&amp; build\bin\axis_engine_tests.exe</x:v>
+        <x:v>cmake --build build --config Debug --target axis_test &amp;&amp; build\bin\axis_test.exe</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -3840,7 +4090,7 @@
         <x:v>tests/unit/test_pathfinding.cpp</x:v>
       </x:c>
       <x:c r="E7" s="9" t="str">
-        <x:v>cmake --build build --config Debug --target axis_engine_tests &amp;&amp; build\bin\axis_engine_tests.exe</x:v>
+        <x:v>cmake --build build --config Debug --target axis_test &amp;&amp; build\bin\axis_test.exe</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -3857,7 +4107,7 @@
         <x:v>tests/unit/test_pathfinding.cpp</x:v>
       </x:c>
       <x:c r="E8" s="9" t="str">
-        <x:v>cmake --build build --config Debug --target axis_engine_tests &amp;&amp; build\bin\axis_engine_tests.exe</x:v>
+        <x:v>cmake --build build --config Debug --target axis_test &amp;&amp; build\bin\axis_test.exe</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -3874,7 +4124,7 @@
         <x:v>tests/unit/test_pathfinding.cpp</x:v>
       </x:c>
       <x:c r="E9" s="9" t="str">
-        <x:v>cmake --build build --config Debug --target axis_engine_tests &amp;&amp; build\bin\axis_engine_tests.exe</x:v>
+        <x:v>cmake --build build --config Debug --target axis_test &amp;&amp; build\bin\axis_test.exe</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -3891,7 +4141,7 @@
         <x:v>tests/unit/test_pathfinding.cpp</x:v>
       </x:c>
       <x:c r="E10" s="9" t="str">
-        <x:v>cmake --build build --config Debug --target axis_engine_tests &amp;&amp; build\bin\axis_engine_tests.exe</x:v>
+        <x:v>cmake --build build --config Debug --target axis_test &amp;&amp; build\bin\axis_test.exe</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -3908,7 +4158,7 @@
         <x:v>tests/unit/test_pathfinding.cpp</x:v>
       </x:c>
       <x:c r="E11" s="9" t="str">
-        <x:v>cmake --build build --config Debug --target axis_engine_tests &amp;&amp; build\bin\axis_engine_tests.exe</x:v>
+        <x:v>cmake --build build --config Debug --target axis_test &amp;&amp; build\bin\axis_test.exe</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -3925,7 +4175,7 @@
         <x:v>tests/unit/test_pathfinding.cpp</x:v>
       </x:c>
       <x:c r="E12" s="9" t="str">
-        <x:v>cmake --build build --config Debug --target axis_engine_tests &amp;&amp; build\bin\axis_engine_tests.exe</x:v>
+        <x:v>cmake --build build --config Debug --target axis_test &amp;&amp; build\bin\axis_test.exe</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -3942,7 +4192,7 @@
         <x:v>tests/unit/test_collision_matrix.cpp</x:v>
       </x:c>
       <x:c r="E13" s="9" t="str">
-        <x:v>cmake --build build --config Debug --target axis_engine_tests &amp;&amp; build\bin\axis_engine_tests.exe</x:v>
+        <x:v>cmake --build build --config Debug --target axis_test &amp;&amp; build\bin\axis_test.exe</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -3959,7 +4209,7 @@
         <x:v>tests/unit/test_collision_matrix.cpp</x:v>
       </x:c>
       <x:c r="E14" s="9" t="str">
-        <x:v>cmake --build build --config Debug --target axis_engine_tests &amp;&amp; build\bin\axis_engine_tests.exe</x:v>
+        <x:v>cmake --build build --config Debug --target axis_test &amp;&amp; build\bin\axis_test.exe</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -3976,7 +4226,7 @@
         <x:v>tests/unit/test_collision_matrix.cpp</x:v>
       </x:c>
       <x:c r="E15" s="9" t="str">
-        <x:v>cmake --build build --config Debug --target axis_engine_tests &amp;&amp; build\bin\axis_engine_tests.exe</x:v>
+        <x:v>cmake --build build --config Debug --target axis_test &amp;&amp; build\bin\axis_test.exe</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -3993,7 +4243,7 @@
         <x:v>tests/unit/test_collision_matrix.cpp</x:v>
       </x:c>
       <x:c r="E16" s="9" t="str">
-        <x:v>cmake --build build --config Debug --target axis_engine_tests &amp;&amp; build\bin\axis_engine_tests.exe</x:v>
+        <x:v>cmake --build build --config Debug --target axis_test &amp;&amp; build\bin\axis_test.exe</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -4010,7 +4260,7 @@
         <x:v>tests/unit/test_entity_manager.cpp</x:v>
       </x:c>
       <x:c r="E17" s="9" t="str">
-        <x:v>cmake --build build --config Debug --target axis_engine_tests &amp;&amp; build\bin\axis_engine_tests.exe</x:v>
+        <x:v>cmake --build build --config Debug --target axis_test &amp;&amp; build\bin\axis_test.exe</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -4027,7 +4277,7 @@
         <x:v>tests/unit/test_entity_manager.cpp</x:v>
       </x:c>
       <x:c r="E18" s="9" t="str">
-        <x:v>cmake --build build --config Debug --target axis_engine_tests &amp;&amp; build\bin\axis_engine_tests.exe</x:v>
+        <x:v>cmake --build build --config Debug --target axis_test &amp;&amp; build\bin\axis_test.exe</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -4044,7 +4294,7 @@
         <x:v>tests/unit/test_entity_manager.cpp</x:v>
       </x:c>
       <x:c r="E19" s="9" t="str">
-        <x:v>cmake --build build --config Debug --target axis_engine_tests &amp;&amp; build\bin\axis_engine_tests.exe</x:v>
+        <x:v>cmake --build build --config Debug --target axis_test &amp;&amp; build\bin\axis_test.exe</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -4061,7 +4311,7 @@
         <x:v>tests/unit/test_entity_manager.cpp</x:v>
       </x:c>
       <x:c r="E20" s="9" t="str">
-        <x:v>cmake --build build --config Debug --target axis_engine_tests &amp;&amp; build\bin\axis_engine_tests.exe</x:v>
+        <x:v>cmake --build build --config Debug --target axis_test &amp;&amp; build\bin\axis_test.exe</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -4078,7 +4328,7 @@
         <x:v>tests/unit/test_entity_manager.cpp</x:v>
       </x:c>
       <x:c r="E21" s="9" t="str">
-        <x:v>cmake --build build --config Debug --target axis_engine_tests &amp;&amp; build\bin\axis_engine_tests.exe</x:v>
+        <x:v>cmake --build build --config Debug --target axis_test &amp;&amp; build\bin\axis_test.exe</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -4095,7 +4345,7 @@
         <x:v>tests/unit/test_entity_manager.cpp</x:v>
       </x:c>
       <x:c r="E22" s="9" t="str">
-        <x:v>cmake --build build --config Debug --target axis_engine_tests &amp;&amp; build\bin\axis_engine_tests.exe</x:v>
+        <x:v>cmake --build build --config Debug --target axis_test &amp;&amp; build\bin\axis_test.exe</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -4112,7 +4362,7 @@
         <x:v>tests/integration/test_transform_system.cpp</x:v>
       </x:c>
       <x:c r="E23" s="9" t="str">
-        <x:v>cmake --build build --config Debug --target axis_engine_tests &amp;&amp; build\bin\axis_engine_tests.exe</x:v>
+        <x:v>cmake --build build --config Debug --target axis_test &amp;&amp; build\bin\axis_test.exe</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -4129,7 +4379,7 @@
         <x:v>tests/integration/test_transform_system.cpp</x:v>
       </x:c>
       <x:c r="E24" s="9" t="str">
-        <x:v>cmake --build build --config Debug --target axis_engine_tests &amp;&amp; build\bin\axis_engine_tests.exe</x:v>
+        <x:v>cmake --build build --config Debug --target axis_test &amp;&amp; build\bin\axis_test.exe</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -4146,7 +4396,7 @@
         <x:v>tests/integration/test_transform_system.cpp</x:v>
       </x:c>
       <x:c r="E25" s="9" t="str">
-        <x:v>cmake --build build --config Debug --target axis_engine_tests &amp;&amp; build\bin\axis_engine_tests.exe</x:v>
+        <x:v>cmake --build build --config Debug --target axis_test &amp;&amp; build\bin\axis_test.exe</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -4163,7 +4413,109 @@
         <x:v>tests/integration/test_transform_system.cpp</x:v>
       </x:c>
       <x:c r="E26" s="9" t="str">
-        <x:v>cmake --build build --config Debug --target axis_engine_tests &amp;&amp; build\bin\axis_engine_tests.exe</x:v>
+        <x:v>cmake --build build --config Debug --target axis_test &amp;&amp; build\bin\axis_test.exe</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="28.5" customHeight="1">
+      <x:c r="A27" t="str">
+        <x:v>EV-001</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>Core/EventManager</x:v>
+      </x:c>
+      <x:c r="C27" s="8" t="str">
+        <x:v>Generic unsubscribe removes listener across event dispatchers</x:v>
+      </x:c>
+      <x:c r="D27" s="8" t="str">
+        <x:v>tests/unit/test_event_manager.cpp</x:v>
+      </x:c>
+      <x:c r="E27" s="8" t="str">
+        <x:v>cmake --build build --config Debug --target axis_test &amp;&amp; build\bin\axis_test.exe</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="28.5" customHeight="1">
+      <x:c r="A28" t="str">
+        <x:v>EV-002</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>Core/EventSubscriptionList</x:v>
+      </x:c>
+      <x:c r="C28" s="8" t="str">
+        <x:v>Subscription list clears mixed event types</x:v>
+      </x:c>
+      <x:c r="D28" s="8" t="str">
+        <x:v>tests/unit/test_event_manager.cpp</x:v>
+      </x:c>
+      <x:c r="E28" s="8" t="str">
+        <x:v>cmake --build build --config Debug --target axis_test &amp;&amp; build\bin\axis_test.exe</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="28.5" customHeight="1">
+      <x:c r="A29" t="str">
+        <x:v>TX-001</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>Render/Texture</x:v>
+      </x:c>
+      <x:c r="C29" s="8" t="str">
+        <x:v>Pixel data ownership survives value copies</x:v>
+      </x:c>
+      <x:c r="D29" s="8" t="str">
+        <x:v>tests/unit/test_texture_ownership.cpp</x:v>
+      </x:c>
+      <x:c r="E29" s="8" t="str">
+        <x:v>cmake --build build --config Debug --target axis_test &amp;&amp; build\bin\axis_test.exe</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="28.5" customHeight="1">
+      <x:c r="A30" t="str">
+        <x:v>TX-002</x:v>
+      </x:c>
+      <x:c r="B30" t="str">
+        <x:v>Render/Texture</x:v>
+      </x:c>
+      <x:c r="C30" s="8" t="str">
+        <x:v>Pixel data ownership survives vector reallocation</x:v>
+      </x:c>
+      <x:c r="D30" s="8" t="str">
+        <x:v>tests/unit/test_texture_ownership.cpp</x:v>
+      </x:c>
+      <x:c r="E30" s="8" t="str">
+        <x:v>cmake --build build --config Debug --target axis_test &amp;&amp; build\bin\axis_test.exe</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="28.5" customHeight="1">
+      <x:c r="A31" t="str">
+        <x:v>TX-003</x:v>
+      </x:c>
+      <x:c r="B31" t="str">
+        <x:v>Resource/TextureManager</x:v>
+      </x:c>
+      <x:c r="C31" s="8" t="str">
+        <x:v>Unload releases kept CPU pixel data</x:v>
+      </x:c>
+      <x:c r="D31" s="8" t="str">
+        <x:v>tests/unit/test_texture_ownership.cpp</x:v>
+      </x:c>
+      <x:c r="E31" s="8" t="str">
+        <x:v>cmake --build build --config Debug --target axis_test &amp;&amp; build\bin\axis_test.exe</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="28.5" customHeight="1">
+      <x:c r="A32" t="str">
+        <x:v>BS-001</x:v>
+      </x:c>
+      <x:c r="B32" t="str">
+        <x:v>Scene/BinarySceneSerializer</x:v>
+      </x:c>
+      <x:c r="C32" s="8" t="str">
+        <x:v>Binary serializer v3 round-trips config and material fields</x:v>
+      </x:c>
+      <x:c r="D32" s="8" t="str">
+        <x:v>tests/integration/test_binary_scene_serializer.cpp</x:v>
+      </x:c>
+      <x:c r="E32" s="8" t="str">
+        <x:v>cmake --build build --config Debug --target axis_test &amp;&amp; build\bin\axis_test.exe</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>